<commit_message>
WIP identified relations issues
</commit_message>
<xml_diff>
--- a/Tests/Failing Structures test.xlsx
+++ b/Tests/Failing Structures test.xlsx
@@ -5,17 +5,18 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://queensuca-my.sharepoint.com/personal/gs13_queensu_ca/Documents/Python/Projects/StructureRelations/tests/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\OneDrive - Queen's University\Python\Projects\StructureRelations\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{2C35C163-7C59-4824-9564-26E1499506B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CD314B4D-DA7E-4C46-BDDD-AA85215B965F}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FFE1C8E-0C39-4FB9-8FB4-5F0A741EDCED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="13740" windowHeight="21120" firstSheet="1" activeTab="2" xr2:uid="{812813CE-6446-4909-B9E6-F7875269C392}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{812813CE-6446-4909-B9E6-F7875269C392}"/>
   </bookViews>
   <sheets>
     <sheet name="Relationship Diagram" sheetId="2" r:id="rId1"/>
     <sheet name="Structure Summary" sheetId="3" r:id="rId2"/>
     <sheet name="Relationship Matrix" sheetId="1" r:id="rId3"/>
+    <sheet name="Slice Relationships" sheetId="5" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="73">
   <si>
     <t>Structure</t>
   </si>
@@ -209,6 +210,54 @@
   </si>
   <si>
     <t>D:\OneDrive - Queen's University\Python\Projects\StructureRelations\tests\RS.CNS_FSRT_2_GTV.BRAI.dcm</t>
+  </si>
+  <si>
+    <t>Slice Start</t>
+  </si>
+  <si>
+    <t>Slice End</t>
+  </si>
+  <si>
+    <t>Boundary</t>
+  </si>
+  <si>
+    <t>a_present</t>
+  </si>
+  <si>
+    <t>b_present</t>
+  </si>
+  <si>
+    <t>slice_relation_type</t>
+  </si>
+  <si>
+    <t>slice_de27im_bits</t>
+  </si>
+  <si>
+    <t>cumulative_relation_type</t>
+  </si>
+  <si>
+    <t>slice_index</t>
+  </si>
+  <si>
+    <t>NaN</t>
+  </si>
+  <si>
+    <t>CONTAINS</t>
+  </si>
+  <si>
+    <t>OVERLAPS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">011001001000000000000000000	</t>
+  </si>
+  <si>
+    <t>111001001111001001111001001</t>
+  </si>
+  <si>
+    <t>000001111000000000000000000</t>
+  </si>
+  <si>
+    <t>Boundary2</t>
   </si>
 </sst>
 </file>
@@ -216,9 +265,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -241,13 +290,31 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="3">
@@ -277,29 +344,44 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="3" fillId="2" borderId="0" xfId="2" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="2"/>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="0" xfId="2" quotePrefix="1" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Bad" xfId="2" builtinId="27"/>
     <cellStyle name="Heading 1" xfId="1" builtinId="16"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="2">
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -401,6 +483,34 @@
     <tableColumn id="2" xr3:uid="{5B4406BA-5524-43DF-9C8B-B54A27130DB5}" name="B"/>
     <tableColumn id="3" xr3:uid="{E4EBD421-309E-4711-A033-64FBF35C37E9}" name="Expected"/>
     <tableColumn id="4" xr3:uid="{DC63C837-2715-479A-9AFA-C84F27FAA185}" name="Actual"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4E0B2EF7-7D9F-4DD4-ACFB-3B1549232740}" name="Table4" displayName="Table4" ref="A1:F16" totalsRowShown="0">
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{873F0775-6424-4631-99BD-BCCE08C41164}" name="slice_index" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{ED49B1F8-BCAB-4947-A304-D913DDA65C73}" name="a_present"/>
+    <tableColumn id="3" xr3:uid="{BCEA8CFA-6BF4-4BC2-9643-096DA5141D70}" name="b_present"/>
+    <tableColumn id="4" xr3:uid="{C0D85F29-259B-4EED-BE64-8177399BC3DA}" name="slice_relation_type"/>
+    <tableColumn id="5" xr3:uid="{65811AC3-4ED3-4C22-AC89-2A3D11A120D5}" name="slice_de27im_bits" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{0DFDADCA-2614-4FBB-AFD4-DAC006E9C8C2}" name="cumulative_relation_type"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9FDAAFF3-021C-4AC7-9960-21B7ADABBE55}" name="Table5" displayName="Table5" ref="I1:N6" totalsRowShown="0">
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{E0803622-65C4-4299-B9EB-1B4BECE08F7C}" name="Structure ID"/>
+    <tableColumn id="2" xr3:uid="{69C30637-0E09-491A-A3A3-25E20FCA3788}" name="# Regions"/>
+    <tableColumn id="3" xr3:uid="{DB81C63A-6C6A-452D-98AE-C321EFD869DF}" name="Slice Start"/>
+    <tableColumn id="4" xr3:uid="{71768FAC-1E02-4B38-BA82-2D99FA39E135}" name="Slice End"/>
+    <tableColumn id="5" xr3:uid="{BC262651-39F8-451D-B5AB-569E045425A9}" name="Boundary"/>
+    <tableColumn id="6" xr3:uid="{F7857836-8798-4A35-9EEA-90A6259ACF32}" name="Boundary2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -727,28 +837,28 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="3:10" ht="20.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
     </row>
     <row r="3" spans="3:10" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
-      <c r="J3" s="3"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
+      <c r="I3" s="5"/>
+      <c r="J3" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -775,15 +885,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="20.25" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
     </row>
     <row r="2" spans="1:7" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
@@ -824,7 +934,7 @@
       <c r="E3">
         <v>1</v>
       </c>
-      <c r="F3" s="5">
+      <c r="F3" s="3">
         <v>8720.42</v>
       </c>
       <c r="G3" t="s">
@@ -847,7 +957,7 @@
       <c r="E4">
         <v>1</v>
       </c>
-      <c r="F4" s="5">
+      <c r="F4" s="3">
         <v>1444.9</v>
       </c>
       <c r="G4" t="s">
@@ -870,7 +980,7 @@
       <c r="E5">
         <v>1</v>
       </c>
-      <c r="F5" s="5">
+      <c r="F5" s="3">
         <v>1417.46</v>
       </c>
       <c r="G5" t="s">
@@ -893,7 +1003,7 @@
       <c r="E6">
         <v>2</v>
       </c>
-      <c r="F6" s="4">
+      <c r="F6" s="2">
         <v>29.98</v>
       </c>
       <c r="G6" t="s">
@@ -916,7 +1026,7 @@
       <c r="E7">
         <v>1</v>
       </c>
-      <c r="F7" s="4">
+      <c r="F7" s="2">
         <v>29.83</v>
       </c>
       <c r="G7" t="s">
@@ -939,7 +1049,7 @@
       <c r="E8">
         <v>1</v>
       </c>
-      <c r="F8" s="4">
+      <c r="F8" s="2">
         <v>27.99</v>
       </c>
       <c r="G8" t="s">
@@ -1097,7 +1207,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5CE839A-FD31-434C-95D0-5778417B8A6C}">
-  <dimension ref="A1:M16"/>
+  <dimension ref="A1:U16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
@@ -1108,9 +1218,14 @@
     <col min="10" max="11" width="13.5703125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="13.5703125" customWidth="1"/>
     <col min="13" max="13" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="20" max="21" width="9.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1144,8 +1259,26 @@
       <c r="M1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="P1" t="s">
+        <v>48</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>53</v>
+      </c>
+      <c r="R1" t="s">
+        <v>57</v>
+      </c>
+      <c r="S1" t="s">
+        <v>58</v>
+      </c>
+      <c r="T1" t="s">
+        <v>59</v>
+      </c>
+      <c r="U1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -1179,8 +1312,23 @@
       <c r="M2" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="P2" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q2">
+        <v>1</v>
+      </c>
+      <c r="R2">
+        <v>-1.3</v>
+      </c>
+      <c r="S2">
+        <v>-0.1</v>
+      </c>
+      <c r="U2">
+        <v>-0.05</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -1214,8 +1362,23 @@
       <c r="M3" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="P3" t="s">
+        <v>2</v>
+      </c>
+      <c r="Q3">
+        <v>1</v>
+      </c>
+      <c r="R3">
+        <v>-1.1000000000000001</v>
+      </c>
+      <c r="S3">
+        <v>-0.3</v>
+      </c>
+      <c r="U3">
+        <v>-0.25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1249,8 +1412,20 @@
       <c r="M4" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="P4" t="s">
+        <v>6</v>
+      </c>
+      <c r="Q4">
+        <v>2</v>
+      </c>
+      <c r="R4">
+        <v>-1.3</v>
+      </c>
+      <c r="S4">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -1284,8 +1459,20 @@
       <c r="M5" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="P5" t="s">
+        <v>4</v>
+      </c>
+      <c r="Q5">
+        <v>1</v>
+      </c>
+      <c r="R5">
+        <v>-0.5</v>
+      </c>
+      <c r="S5">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -1319,8 +1506,23 @@
       <c r="M6" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="P6" t="s">
+        <v>1</v>
+      </c>
+      <c r="Q6">
+        <v>1</v>
+      </c>
+      <c r="R6">
+        <v>-0.3</v>
+      </c>
+      <c r="S6">
+        <v>0.6</v>
+      </c>
+      <c r="T6">
+        <v>-0.35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -1355,7 +1557,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="J8" t="s">
         <v>4</v>
       </c>
@@ -1369,7 +1571,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="J9" t="s">
         <v>4</v>
       </c>
@@ -1383,7 +1585,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="J10" t="s">
         <v>4</v>
       </c>
@@ -1397,7 +1599,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="J11" t="s">
         <v>5</v>
       </c>
@@ -1411,7 +1613,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="J12" t="s">
         <v>5</v>
       </c>
@@ -1425,7 +1627,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="J13" t="s">
         <v>5</v>
       </c>
@@ -1439,7 +1641,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="J14" t="s">
         <v>3</v>
       </c>
@@ -1453,7 +1655,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="J15" t="s">
         <v>3</v>
       </c>
@@ -1467,7 +1669,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="J16" t="s">
         <v>1</v>
       </c>
@@ -1489,4 +1691,438 @@
     <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFBA188C-15AB-41FE-B793-CC6FB692AE47}">
+  <dimension ref="A1:N16"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.85546875" customWidth="1"/>
+    <col min="2" max="3" width="11.7109375" customWidth="1"/>
+    <col min="4" max="4" width="19.42578125" customWidth="1"/>
+    <col min="5" max="5" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5703125" customWidth="1"/>
+    <col min="11" max="11" width="11.7109375" customWidth="1"/>
+    <col min="12" max="12" width="11" customWidth="1"/>
+    <col min="13" max="13" width="11.5703125" customWidth="1"/>
+    <col min="14" max="14" width="12.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E1" t="s">
+        <v>63</v>
+      </c>
+      <c r="F1" t="s">
+        <v>64</v>
+      </c>
+      <c r="I1" t="s">
+        <v>48</v>
+      </c>
+      <c r="J1" t="s">
+        <v>53</v>
+      </c>
+      <c r="K1" t="s">
+        <v>57</v>
+      </c>
+      <c r="L1" t="s">
+        <v>58</v>
+      </c>
+      <c r="M1" t="s">
+        <v>59</v>
+      </c>
+      <c r="N1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" s="8">
+        <v>-0.35</v>
+      </c>
+      <c r="B2" t="b">
+        <v>1</v>
+      </c>
+      <c r="C2" t="b">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="F2" t="s">
+        <v>66</v>
+      </c>
+      <c r="I2" t="s">
+        <v>5</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2">
+        <v>-1.3</v>
+      </c>
+      <c r="L2">
+        <v>-0.1</v>
+      </c>
+      <c r="N2" s="6">
+        <v>-0.05</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" s="8">
+        <v>-0.3</v>
+      </c>
+      <c r="B3" t="b">
+        <v>1</v>
+      </c>
+      <c r="C3" t="b">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>67</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="F3" t="s">
+        <v>67</v>
+      </c>
+      <c r="I3" t="s">
+        <v>2</v>
+      </c>
+      <c r="J3">
+        <v>1</v>
+      </c>
+      <c r="K3">
+        <v>-1.1000000000000001</v>
+      </c>
+      <c r="L3">
+        <v>-0.3</v>
+      </c>
+      <c r="N3">
+        <v>-0.25</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" s="8">
+        <v>-0.25</v>
+      </c>
+      <c r="B4" t="b">
+        <v>1</v>
+      </c>
+      <c r="C4" t="b">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s">
+        <v>67</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="F4" t="s">
+        <v>67</v>
+      </c>
+      <c r="I4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J4">
+        <v>2</v>
+      </c>
+      <c r="K4">
+        <v>-1.3</v>
+      </c>
+      <c r="L4">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" s="8">
+        <v>-0.2</v>
+      </c>
+      <c r="B5" t="b">
+        <v>1</v>
+      </c>
+      <c r="C5" t="b">
+        <v>1</v>
+      </c>
+      <c r="D5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="F5" t="s">
+        <v>67</v>
+      </c>
+      <c r="I5" t="s">
+        <v>4</v>
+      </c>
+      <c r="J5">
+        <v>1</v>
+      </c>
+      <c r="K5">
+        <v>-0.5</v>
+      </c>
+      <c r="L5">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" s="8">
+        <v>-0.1</v>
+      </c>
+      <c r="B6" t="b">
+        <v>1</v>
+      </c>
+      <c r="C6" t="b">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
+        <v>67</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="F6" t="s">
+        <v>67</v>
+      </c>
+      <c r="I6" t="s">
+        <v>1</v>
+      </c>
+      <c r="J6">
+        <v>1</v>
+      </c>
+      <c r="K6">
+        <v>-0.3</v>
+      </c>
+      <c r="L6">
+        <v>0.6</v>
+      </c>
+      <c r="M6">
+        <v>-0.35</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7" s="9">
+        <v>-0.05</v>
+      </c>
+      <c r="B7" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="C7" s="10" t="b">
+        <v>1</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" s="8">
+        <v>0</v>
+      </c>
+      <c r="B8" t="b">
+        <v>1</v>
+      </c>
+      <c r="C8" t="b">
+        <v>1</v>
+      </c>
+      <c r="D8" t="s">
+        <v>67</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="F8" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" s="8">
+        <v>0.1</v>
+      </c>
+      <c r="B9" t="b">
+        <v>1</v>
+      </c>
+      <c r="C9" t="b">
+        <v>1</v>
+      </c>
+      <c r="D9" t="s">
+        <v>67</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="F9" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10" s="8">
+        <v>0.2</v>
+      </c>
+      <c r="B10" t="b">
+        <v>1</v>
+      </c>
+      <c r="C10" t="b">
+        <v>1</v>
+      </c>
+      <c r="D10" t="s">
+        <v>67</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="F10" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11" s="8">
+        <v>0.3</v>
+      </c>
+      <c r="B11" t="b">
+        <v>1</v>
+      </c>
+      <c r="C11" t="b">
+        <v>1</v>
+      </c>
+      <c r="D11" t="s">
+        <v>67</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="F11" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A12" s="8">
+        <v>0.4</v>
+      </c>
+      <c r="B12" t="b">
+        <v>1</v>
+      </c>
+      <c r="C12" t="b">
+        <v>1</v>
+      </c>
+      <c r="D12" t="s">
+        <v>67</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="F12" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13" s="8">
+        <v>0.45</v>
+      </c>
+      <c r="B13" t="b">
+        <v>1</v>
+      </c>
+      <c r="C13" t="b">
+        <v>1</v>
+      </c>
+      <c r="D13" t="s">
+        <v>67</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="F13" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A14" s="8">
+        <v>0.5</v>
+      </c>
+      <c r="B14" t="b">
+        <v>1</v>
+      </c>
+      <c r="C14" t="b">
+        <v>1</v>
+      </c>
+      <c r="D14" t="s">
+        <v>67</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="F14" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A15" s="8">
+        <v>0.6</v>
+      </c>
+      <c r="B15" t="b">
+        <v>1</v>
+      </c>
+      <c r="C15" t="b">
+        <v>1</v>
+      </c>
+      <c r="D15" t="s">
+        <v>67</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="F15" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A16" s="8">
+        <v>0.65</v>
+      </c>
+      <c r="B16" t="b">
+        <v>1</v>
+      </c>
+      <c r="C16" t="b">
+        <v>1</v>
+      </c>
+      <c r="D16" t="s">
+        <v>66</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="F16" t="s">
+        <v>68</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="2">
+    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>